<commit_message>
LØM-app 2.18.0: v7.3 for alle 91 økter, SOFT og leteskjema i MA03/MA10, muntlig eksamen og Eksamen på tvers
</commit_message>
<xml_diff>
--- a/pensum/ma06/MA06_Produkt_Oppgaver_v6.xlsx
+++ b/pensum/ma06/MA06_Produkt_Oppgaver_v6.xlsx
@@ -824,7 +824,7 @@
     <t xml:space="preserve">1B g) Pakken</t>
   </si>
   <si>
-    <t xml:space="preserve">Tilleggene koster 295 kr per jobb, lite mot 1 075 kr i forskjell hos Lunde. De skal stå i tilbudet med navn, og garantien må si hva den gir ut over loven</t>
+    <t xml:space="preserve">Tilleggene koster 295 kr per jobb, lite mot 1 075 kr i forskjell hos familien Moen. De skal stå i tilbudet med navn, og garantien må si hva den gir ut over loven</t>
   </si>
   <si>
     <t xml:space="preserve">1C Summene i tabellen</t>
@@ -1578,7 +1578,7 @@
         <v>1</v>
       </c>
     </row>
-    <row ht="17.25" customHeight="true" r="5" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="3" t="s">
         <v>2</v>
       </c>
@@ -1603,42 +1603,42 @@
         <v>6</v>
       </c>
     </row>
-    <row ht="17.25" customHeight="true" r="11" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row ht="17.25" customHeight="true" r="12" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row ht="17.25" customHeight="true" r="13" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row ht="17.25" customHeight="true" r="14" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row ht="17.25" customHeight="true" r="15" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B15" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row ht="17.25" customHeight="true" r="16" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row ht="17.25" customHeight="true" r="17" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row ht="17.25" customHeight="true" r="18" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="2" t="s">
         <v>14</v>
       </c>
@@ -1973,7 +1973,7 @@
         <v>Skriv svaret i den gule cellen.</v>
       </c>
     </row>
-    <row ht="46.5" customHeight="true" r="30" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="14" t="s">
         <v>49</v>
       </c>
@@ -1983,7 +1983,7 @@
         <v>Velg i nedtrekksmenyen.</v>
       </c>
     </row>
-    <row ht="17.25" customHeight="true" r="32" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B32" s="9" t="s">
         <v>50</v>
       </c>
@@ -2406,7 +2406,7 @@
         <v>71</v>
       </c>
     </row>
-    <row ht="60.75" customHeight="true" r="20" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="9" t="s">
         <v>72</v>
       </c>
@@ -2545,7 +2545,7 @@
         <v>Skriv svaret i den gule cellen.</v>
       </c>
     </row>
-    <row ht="46.5" customHeight="true" r="35" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B35" s="14" t="s">
         <v>86</v>
       </c>
@@ -2600,7 +2600,7 @@
         <v>Velg i nedtrekksmenyen.</v>
       </c>
     </row>
-    <row ht="17.25" customHeight="true" r="43" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B43" s="9" t="s">
         <v>92</v>
       </c>
@@ -2636,7 +2636,7 @@
     </row>
     <row r="47" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B47" s="21" t="str">
-        <f aca="false">IF(LEN(B44)&lt;40,"",IF(AND(ISNUMBER(SEARCH("295",B44)),ISNUMBER(SEARCH("tilbud",B44))),"Bra: du bruker kostnaden 295 kr per jobb og sier at tilleggene skal stå i tilbudet. Det er slik det utvidete produktet blir synlig.",IF(OR(ISNUMBER(SEARCH("295",B44)),ISNUMBER(SEARCH("tilbud",B44))),"Du er på sporet. Ta med tallet 295 kr per jobb, og si hvor kunden skal se tilleggene: i tilbudet, med navn.","Tips: tilleggene koster 295 kr per jobb, mot 1 075 kr i forskjell hos familien Lunde. Skal de inn, må de stå i tilbudet med navn, og garantien må si hva den gir ut over loven.")))</f>
+        <f aca="false">IF(LEN(B44)&lt;40,"",IF(AND(ISNUMBER(SEARCH("295",B44)),ISNUMBER(SEARCH("tilbud",B44))),"Bra: du bruker kostnaden 295 kr per jobb og sier at tilleggene skal stå i tilbudet. Det er slik det utvidete produktet blir synlig.",IF(OR(ISNUMBER(SEARCH("295",B44)),ISNUMBER(SEARCH("tilbud",B44))),"Du er på sporet. Ta med tallet 295 kr per jobb, og si hvor kunden skal se tilleggene: i tilbudet, med navn.","Tips: tilleggene koster 295 kr per jobb, mot 1 075 kr i forskjell hos familien Moen. Skal de inn, må de stå i tilbudet med navn, og garantien må si hva den gir ut over loven.")))</f>
         <v/>
       </c>
       <c r="C47" s="21"/>
@@ -3737,7 +3737,7 @@
         <v>137</v>
       </c>
     </row>
-    <row ht="60.75" customHeight="true" r="17" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="9" t="s">
         <v>147</v>
       </c>
@@ -3979,7 +3979,7 @@
         <v>135</v>
       </c>
     </row>
-    <row ht="17.25" customHeight="true" r="39" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B39" s="9" t="s">
         <v>164</v>
       </c>
@@ -4499,7 +4499,7 @@
       <c r="F20" s="8"/>
       <c r="G20" s="8"/>
     </row>
-    <row ht="60.75" customHeight="true" r="21" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B21" s="9" t="s">
         <v>189</v>
       </c>
@@ -4603,7 +4603,7 @@
         <v>Velg i nedtrekksmenyen.</v>
       </c>
     </row>
-    <row ht="17.25" customHeight="true" r="35" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B35" s="9" t="s">
         <v>201</v>
       </c>
@@ -5031,7 +5031,7 @@
       <c r="F18" s="8"/>
       <c r="G18" s="8"/>
     </row>
-    <row ht="60.75" customHeight="true" r="19" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B19" s="9" t="s">
         <v>219</v>
       </c>

</xml_diff>